<commit_message>
Add Paper Mill Rd to vacant set and switch map to satellite view
- Include 2500 Paper Mill Rd, Mobile AL as the 9th vacant property
  in both the spreadsheet and the map.
- Map now uses Esri World Imagery (satellite) with a place-label
  overlay and a layers toggle for satellite/street views.

https://claude.ai/code/session_01Tsi18E6iYrAkqhnRUyuvNs
</commit_message>
<xml_diff>
--- a/CCRE_PORTFOLIO_42026_Vacant_Only.xlsx
+++ b/CCRE_PORTFOLIO_42026_Vacant_Only.xlsx
@@ -825,7 +825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB16"/>
+  <dimension ref="A1:AB17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.28515625" customWidth="1" min="1" max="1"/>
@@ -1830,125 +1830,216 @@
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
+          <t>https://earth.google.com/web/search/2500+Paper+Mill+Rd,+Mobile,+AL/@30.7388799,-88.0533082,13.24312505a,712.04570508d,35y,0h,0t,0r/data=CiwiJgokCQrN9c8Axj9AEZ5APjYiwz9AGThIz8yal1rAIefzT2lcmVrAQgIIATIpCicKJQohMWdTMFZXLWRMNTk0RFVHSzBBazR3alZaVXE5NDhMWGpVIAE6AwoBMEICCABKCAjS3LSqBhAB</t>
+        </is>
+      </c>
+      <c r="C12" s="60" t="inlineStr">
+        <is>
+          <t>2500 Paper Mill Rd</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="F12" s="71" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fi/l5fmb0aodhtzmi44he5ri/2500-Paper-Mill-Flyer.pdf?rlkey=sb7zrdw0xxqacfd32wigj9yvi&amp;st=r2fncf98&amp;dl=0</t>
+        </is>
+      </c>
+      <c r="G12" s="28">
+        <f>(H21/(I21*43560))</f>
+        <v/>
+      </c>
+      <c r="H12" s="79" t="n">
+        <v>19786</v>
+      </c>
+      <c r="I12" s="49" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="J12" s="69" t="inlineStr">
+        <is>
+          <t>https://www.dropbox.com/scl/fi/w8spszhvwv6idsbszg9a4/012-Univar-Kenobi-Portfolio-Paper-Mill-Rd.-Mobile-AL.pdf?rlkey=rfuwjx3amwx57g6p6tud318lf&amp;st=cmfc5ctz&amp;dl=0</t>
+        </is>
+      </c>
+      <c r="K12" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industrial </t>
+        </is>
+      </c>
+      <c r="L12" s="27" t="inlineStr">
+        <is>
+          <t>I-2 Heavy Industrial</t>
+        </is>
+      </c>
+      <c r="M12" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Occupied </t>
+        </is>
+      </c>
+      <c r="N12" s="27" t="inlineStr">
+        <is>
+          <t>Vacant</t>
+        </is>
+      </c>
+      <c r="O12" s="27" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="P12" s="33" t="n">
+        <v>12232.67</v>
+      </c>
+      <c r="Q12" s="33" t="n">
+        <v>12337</v>
+      </c>
+      <c r="R12" s="33" t="n">
+        <v>1066.1</v>
+      </c>
+      <c r="S12" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="80" t="n"/>
+      <c r="U12" s="33" t="n"/>
+      <c r="V12" s="80" t="n"/>
+      <c r="W12" s="66" t="n">
+        <v>46143</v>
+      </c>
+      <c r="X12" s="66" t="n">
+        <v>48091</v>
+      </c>
+      <c r="Y12" s="80" t="inlineStr">
+        <is>
+          <t>4.0% annually</t>
+        </is>
+      </c>
+      <c r="Z12" s="67" t="inlineStr">
+        <is>
+          <t>Two (2) 3-year options to renew at market rent</t>
+        </is>
+      </c>
+      <c r="AA12" s="81" t="n">
+        <v>45940</v>
+      </c>
+    </row>
+    <row r="13" ht="45.6" customFormat="1" customHeight="1" s="12" thickBot="1">
+      <c r="A13" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
           <t>https://earth.google.com/web/search/450+Butler+Drive,+Murfreesboro,+TN/@35.80316366,-86.38932792,194.46627213a,892.36418324d,35y,-0h,0t,0r/data=CiwiJgokCRbbScZdoz1AEUyFr0A0oT1AGRN49Z5_zFfAIfPIePzKzVfAQgIIATIpCicKJQohMWdTMFZXLWRMNTk0RFVHSzBBazR3alZaVXE5NDhMWGpVIAE6AwoBMEICCABKCAjS3LSqBhAB</t>
         </is>
       </c>
-      <c r="C12" s="60" t="inlineStr">
+      <c r="C13" s="60" t="inlineStr">
         <is>
           <t>450 Butler Dr</t>
         </is>
       </c>
-      <c r="D12" s="27" t="inlineStr">
+      <c r="D13" s="27" t="inlineStr">
         <is>
           <t>Murfreesboro</t>
         </is>
       </c>
-      <c r="E12" s="27" t="inlineStr">
+      <c r="E13" s="27" t="inlineStr">
         <is>
           <t>TN</t>
         </is>
       </c>
-      <c r="F12" s="71" t="inlineStr">
+      <c r="F13" s="71" t="inlineStr">
         <is>
           <t>https://www.dropbox.com/scl/fi/5xipkajd3io3g4e36z6wq/450-Butler-Dr-Murfreesboro02.pdf?rlkey=10q621outsl07pbhnv8t06qbm&amp;st=pfnhk4co&amp;dl=0</t>
         </is>
       </c>
-      <c r="G12" s="28">
+      <c r="G13" s="28">
         <f>(H23/(I23*43560))</f>
         <v/>
       </c>
-      <c r="H12" s="79" t="n">
+      <c r="H13" s="79" t="n">
         <v>53750</v>
       </c>
-      <c r="I12" s="49" t="n">
+      <c r="I13" s="49" t="n">
         <v>5.43</v>
       </c>
-      <c r="J12" s="49" t="inlineStr">
+      <c r="J13" s="49" t="inlineStr">
         <is>
           <t>Zoning link</t>
         </is>
       </c>
-      <c r="K12" s="27" t="inlineStr">
+      <c r="K13" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Industrial </t>
         </is>
       </c>
-      <c r="L12" s="27" t="inlineStr">
+      <c r="L13" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">Heavy Industrial </t>
         </is>
       </c>
-      <c r="M12" s="27" t="inlineStr">
+      <c r="M13" s="27" t="inlineStr">
         <is>
           <t>Vacant</t>
         </is>
       </c>
-      <c r="N12" s="27" t="inlineStr">
+      <c r="N13" s="27" t="inlineStr">
         <is>
           <t>Vacant</t>
         </is>
       </c>
-      <c r="O12" s="27" t="inlineStr">
+      <c r="O13" s="27" t="inlineStr">
         <is>
           <t>NNN</t>
         </is>
       </c>
-      <c r="P12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" s="33">
+      <c r="P13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="33">
         <f>H23*T23</f>
         <v/>
       </c>
-      <c r="V12" s="80" t="n"/>
-      <c r="W12" s="80" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X12" s="80" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Y12" s="80" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Z12" s="80" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AA12" s="81" t="n">
+      <c r="V13" s="80" t="n"/>
+      <c r="W13" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="X13" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Y13" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Z13" s="80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AA13" s="81" t="n">
         <v>46112</v>
       </c>
-    </row>
-    <row r="13" ht="45.6" customFormat="1" customHeight="1" s="12" thickBot="1">
-      <c r="B13" s="6" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="82" t="n"/>
-      <c r="T13" s="83" t="n"/>
-      <c r="U13" s="83" t="n"/>
-      <c r="V13" s="83" t="n"/>
-      <c r="W13" s="83" t="n"/>
-      <c r="X13" s="83" t="n"/>
-      <c r="Y13" s="83" t="n"/>
-      <c r="Z13" s="8" t="n"/>
-      <c r="AA13" s="8" t="n"/>
     </row>
     <row r="14" ht="45.6" customFormat="1" customHeight="1" s="12" thickBot="1">
       <c r="B14" s="6" t="n"/>
@@ -1964,40 +2055,52 @@
       <c r="AA14" s="8" t="n"/>
     </row>
     <row r="15" ht="45.6" customFormat="1" customHeight="1" s="12" thickBot="1">
-      <c r="B15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total </t>
-        </is>
-      </c>
-      <c r="C15" s="61">
-        <f>COUNTA(C5:C12)</f>
-        <v/>
-      </c>
-      <c r="G15" s="9">
-        <f>AVERAGE(G5:G12)</f>
-        <v/>
-      </c>
-      <c r="H15" s="82">
-        <f>SUM(H5:H12)</f>
-        <v/>
-      </c>
-      <c r="I15" s="1">
-        <f>SUM(I5:I12)</f>
-        <v/>
-      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="82" t="n"/>
       <c r="T15" s="83" t="n"/>
       <c r="U15" s="83" t="n"/>
       <c r="V15" s="83" t="n"/>
       <c r="W15" s="83" t="n"/>
       <c r="X15" s="83" t="n"/>
       <c r="Y15" s="83" t="n"/>
-      <c r="Z15" s="10" t="n"/>
-      <c r="AA15" s="10" t="n"/>
+      <c r="Z15" s="8" t="n"/>
+      <c r="AA15" s="8" t="n"/>
     </row>
     <row r="16" ht="21.6" customFormat="1" customHeight="1" s="12" thickBot="1">
-      <c r="G16" s="9" t="n"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total </t>
+        </is>
+      </c>
+      <c r="C16" s="61">
+        <f>COUNTA(C5:C13)</f>
+        <v/>
+      </c>
+      <c r="G16" s="9">
+        <f>AVERAGE(G5:G13)</f>
+        <v/>
+      </c>
+      <c r="H16" s="82">
+        <f>SUM(H5:H13)</f>
+        <v/>
+      </c>
+      <c r="I16" s="1">
+        <f>SUM(I5:I13)</f>
+        <v/>
+      </c>
+      <c r="T16" s="83" t="n"/>
+      <c r="U16" s="83" t="n"/>
+      <c r="V16" s="83" t="n"/>
+      <c r="W16" s="83" t="n"/>
+      <c r="X16" s="83" t="n"/>
+      <c r="Y16" s="83" t="n"/>
+      <c r="Z16" s="10" t="n"/>
+      <c r="AA16" s="10" t="n"/>
     </row>
-    <row r="17" ht="45.6" customFormat="1" customHeight="1" s="12" thickBot="1"/>
+    <row r="17" ht="45.6" customFormat="1" customHeight="1" s="12" thickBot="1">
+      <c r="G17" s="9" t="n"/>
+    </row>
     <row r="18" ht="45.6" customFormat="1" customHeight="1" s="12" thickBot="1"/>
     <row r="19" ht="45.6" customFormat="1" customHeight="1" s="12" thickBot="1"/>
     <row r="20" ht="45.6" customFormat="1" customHeight="1" s="12" thickBot="1"/>
@@ -2033,8 +2136,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" display="https://earth.google.com/web/search/6980+Market+Avenue,+El+Paso,+TX/@31.76784607,-106.38254429,1165.63763495a,810.73536689d,35y,-0h,0t,0r/data=CiwiJgokCS8paf5do0FAEcraQzmzokFAGWwebpRZOFTAIQbLfkMzOVTAQgIIATIpCicKJQohMWdTMFZXLWRMNTk0RFVHSzBBazR3alZaVXE5NDhMWGpVIAE6AwoBMEICCABKCAjS3LSqBhAB" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" display="https://earth.google.com/web/search/450+Butler+Drive,+Murfreesboro,+TN/@35.80316366,-86.38932792,194.46627213a,892.36418324d,35y,-0h,0t,0r/data=CiwiJgokCRbbScZdoz1AEUyFr0A0oT1AGRN49Z5_zFfAIfPIePzKzVfAQgIIATIpCicKJQohMWdTMFZXLWRMNTk0RFVHSzBBazR3alZaVXE5NDhMWGpVIAE6AwoBMEICCABKCAjS3LSqBhAB" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" display="https://earth.google.com/web/search/2500+Paper+Mill+Rd,+Mobile,+AL/@30.7388799,-88.0533082,13.24312505a,712.04570508d,35y,0h,0t,0r/data=CiwiJgokCQrN9c8Axj9AEZ5APjYiwz9AGThIz8yal1rAIefzT2lcmVrAQgIIATIpCicKJQohMWdTMFZXLWRMNTk0RFVHSzBBazR3alZaVXE5NDhMWGpVIAE6AwoBMEICCABKCAjS3LSqBhAB" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" display="https://earth.google.com/web/search/450+Butler+Drive,+Murfreesboro,+TN/@35.80316366,-86.38932792,194.46627213a,892.36418324d,35y,-0h,0t,0r/data=CiwiJgokCRbbScZdoz1AEUyFr0A0oT1AGRN49Z5_zFfAIfPIePzKzVfAQgIIATIpCicKJQohMWdTMFZXLWRMNTk0RFVHSzBBazR3alZaVXE5NDhMWGpVIAE6AwoBMEICCABKCAjS3LSqBhAB" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>